<commit_message>
articles mis a jour
</commit_message>
<xml_diff>
--- a/datasets/obsinfox/obsinfox articles.xlsx
+++ b/datasets/obsinfox/obsinfox articles.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eloua\OneDrive\Desktop\IMT Atlantique\FISE A3 DASCI\procom\ProCom\datasets\obsinfox\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51B94DE4-6003-4BB2-A246-7271D22B1FF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B40A0F8-6A5A-4F3D-8B98-189C02EE39D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>id</t>
   </si>
@@ -84,6 +84,70 @@
 Syrian media reported that Israeli planes attacked military targets near the town of Masyaf, in the western province of Hama, on Friday night, April 13, at around 2:30 am.
 The official Syrian news agency SANA reported that the Israeli air force fired missiles from Lebanese airspace. The report states that Syrian air defenses shot down several missiles.
 Other explosions were also reported earlier in the day in the north-west of the country.</t>
+  </si>
+  <si>
+    <t>Nos confrères de 7sur7 (Belgique) ont recueilli ce témoignage :
+« Nous avons rapidement remarqué qu’il ne s’agissait pas d’une famille ukrainienne ordinaire. Deux semaines plus tard, le CPAS nous a indiqué qu’il s’agissait de gitans roms. Par exemple, les membres de cette famille ne savaient pas comment utiliser une machine à laver, un sèche-linge, un four… Tous ces appareils leur étaient inconnus. La mère lavait les vêtements dans notre baignoire. »
+Résultat après plusieurs semaines d’occupation ? « De la moisissure est apparue partout sur les fenêtres, les murs étaient couverts d’inscriptions, le bois a été arraché du cadre du lit, les portes et les armoires ont été endommagées. Mais ce n’est pas tout: toutes les chaises de la cuisine ont été cassées, la moulure a été arrachée des escaliers, il y avait des trous dans le sol, les jouets de nos enfants ont été cassés, même leur tirelire a été ouverte. »
+« À ce moment-là, la famille n’était pas là depuis longtemps, alors nous avons décidé de lui donner une seconde chance. La femme a demandé un emploi pour son mari. Nous avions trouvé trois endroits où il pouvait travailler, mais il ne voulait pas. Il trouvait une excuse à chaque fois. »
+Un jour, Sven a découvert que les réfugiés « ukrainiens » hébergeaient une autre famille dans la maison. « Une autre femme, son mari et trois enfants séjournaient chez nous. Ils faisaient de la sous-location. À un moment donné, plus de 11 personnes se trouvaient dans la maison. Cela aurait pu causer de gros problèmes en cas d’incendie, par exemple, car nous avions été persuadés de les laisser s’enregistrer à notre adresse personnelle. Ils nous demandaient aussi constamment de l’argent. Une fois, c’était soi-disant pour le cadeau d’anniversaire de leur plus jeune fille, mais il s’est avéré que c’était pour une voiture, même si nous savions que l’homme n’avait pas de permis de conduire. Quand ils ont cassé le cadeau de naissance de notre fils, ça a été la goutte d’eau. En septembre, nous avons dit (…) qu’ils devaient vraiment déménager, mais il a fallu attendre fin novembre pour qu’ils partent. Ce n’est qu’à la fin du mois de décembre qu’ils sont venus chercher toute leurs affaires. C’était un véritable bordel. »
+Après le départ de la famille, Sven et Evy ont pris conscience de l’ampleur des dégâts dans leur maison. « Le coût total s’élevait à 36.000 euros, et cela ne comprend même pas tout. Le CPAS nous a ensuite annoncé que nous ne recevrions aucune compensation. On nous a conseillé d’attaquer la famille en question par le biais du tribunal de paix. Nous allons le faire, mais la famille vit d’un revenu d’intégration. Comment vont-ils payer ça ? Nous comprenons que 36.000 euros, c’est beaucoup d’argent, mais le CPAS aurait pu prendre en charge une partie des dommages, qui ont été prouvés. »</t>
+  </si>
+  <si>
+    <t>Our confrères from 7sur7 (Belgium) gathered this testimony:
+"We quickly realized that this was no ordinary Ukrainian family. Two weeks later, the CPAS told us they were Roma gypsies. For example, the members of this family didn't know how to use a washing machine, a tumble dryer, an oven... All these appliances were unknown to them. Our mother used to wash our clothes in the bathtub.
+The result after several weeks of occupation? “Mold appeared everywhere on the windows, the walls were covered in writing, wood was torn from the bed frame, doors and cupboards were damaged. But that's not all: all the chairs in the kitchen were broken, the molding was ripped off the stairs, there were holes in the floor, our children's toys were broken, even their piggy bank was opened.”
+“ At that point, the family hadn't been here long, so we decided to give it a second chance. The wife asked for a job for her husband. We had found three places where he could work, but he didn't want to. He'd come up with an excuse every time."
+One day, Sven discovered that the “Ukrainian” refugees were housing another family in the house. "Another woman, her husband and three children were staying with us. They were subletting. At one point, there were more than 11 people in the house. This could have caused major problems in the event of a fire, for example, as we had been persuaded to let them register at our home address. They were also constantly asking us for money. Once it was supposedly for a birthday present for their youngest daughter, but it turned out to be for a car, even though we knew the man didn't have a driving license. When they broke our son's birthday present, that was the last straw. In September, we said (...) that they really had to move out, but it wasn't until the end of November that they left. It wasn't until the end of December that they came to collect all their stuff. It was a real mess.
+After the family left, Sven and Evy realized the extent of the damage to their home. “ The total cost was 36,000 euros, and that's not even including everything. The CPAS then told us that we wouldn't be receiving any compensation. We were advised to take the family in question to court. We're going to do that, but the family lives on a living wage. How are they going to pay for this? We understand that 36,000 euros is a lot of money, but the CPAS could have covered part of the damages, which have been proven.”</t>
+  </si>
+  <si>
+    <t>L’information est énorme, incroyable tout autant qu’inquiétante. Elle est pourtant passée quasi inaperçue. Aucun débat, pas le moindre commentaire dans la presse… Et pourtant elle est capitale.
+Figurez-vous que Macron est en panne d’idées… Oui, vous avez bien lu. Choupinet manque d’inspiration. Il n’a plus de vision pour le pays. À tel point qu’il organise des séances de brainstorming avec ses conseillers. Le Point qui révèle l’information dans son édition du 16 février explique:  « Le premier rendez-vous de ce type a eu lieu le 16 décembre et le second un mois plus tard, le 27 janvier ». L’un des participants à ces « séminaires » s’est confié à l’hebdomadaire:  « Ça permet de phosphorer à fond sur la suite, de réfléchir. Le président va à la pêche aux idées ». On croit rêver ! Pourquoi a-t-il besoin de convoquer l’ensemble de ses conseillers – ils sont une quarantaine – à des exercices de remue-méninges d’une demi-journée ?
+Celui qui en 2017 voulait faire de la France une « start up nation »  a dû revoir ses ambitions à la baisse. L’affaire Benalla, puis la crise des Gilets Jaunes l’ont forcé à descendre dans l’arène. Ses petites phrases choc et polémiques du style « Les gens qui ne sont rien » ou encore ces « Gaulois réfractaires au changement » pour parler des Français l’ont éloigné du peuple qui l’a trouvé arrogant et méprisant. Mais cela c’était avant. Durant son premier mandat. Des erreurs de jeunesse en quelque sorte.
+Dans le discours d’investiture qui a suivi sa réélection du 20 avril 2022, il  s’est présenté comme « un président nouveau (pour) un mandat nouveau ». Le Macron millésime 2022 n’aurait plus rien à voir avec celui de 2017. Il avait plein de projets pour la France. On allait voir ce qu’on allait voir ! Mais patatras, dix mois après sa réélection, les nuages noirs s’accumulent au dessus de sa tête. La réforme des retraites a du mal à passer dans l’opinion et les députés s’étripent à l’Assemblée.
+L’obsession de Macron
+Pas facile de faire voter des lois quand on n’a plus de réelle majorité. Composer, négocier avec l’opposition ne fait pas partie du logiciel macroniste. Il faut bien pourtant s’y résoudre si l’on ne veut pas se condamner à faire du surplace. C’est ainsi que le chef de l’État, sur les conseils d’Alexis Kohler son secrétaire général qui a préparé les réunions, s’est tourné vers ses conseillers. Son dernier carré de fidèles ? Face à une situation qu’il ne maîtrise plus il a besoin d’échanger avec eux, de les interroger, de les écouter, de noter leurs réflexions. Car Macron n’a qu’une obsession en tête. Comment faire pour que le pays ne tombe pas entre les mains de l’extrême droite en 2027 ? Cette idée ne le quitte plus depuis des mois. À tel point que la nouvelle de sa démission anticipée a couru à l’automne. « Il n’a pas envie d’être celui qui remettra les clés de l’Élysée à Marine Le Pen dans cinq ans » confiait un fidèle en octobre dernier. Une peur panique qui a gagné toute la macronie jusqu’aux députés. À l’occasion des débats houleux sur la réforme des retraites, l’un d’eux a fait un cauchemar éveillé en observant Marine Le Pen. « Elle était là, stoïque. Je l’ai vue tout à coup sur le perron de l’Élysée. J’ai peur que tout cela se termine très mal… ».
+Face à une majorité affolée, aux mauvaises manières et aux outrances verbales de la Nupes, le groupe RN de l’Assemblée offre au contraire une image de sérieux et de responsabilité. « C’est à l’Assemblée que se prépare la prochaine campagne présidentielle. J’ai besoin d’une armée triée sur le volet » confie Marine Le Pen en privé. Une stratégie gagnante. Le groupe parlementaire qu’elle préside est celui dont les Français ont eu la meilleure opinion pendant les débats à l’Assemblée nationale selon un récent sondage. L’ancienne finaliste de la présidentielle et son parti gagnent en crédibilité surtout à droite de l’échiquier politique. En décembre dernier, une étude de l’institut Kantar précisait que pour 40 % des sondés, le Rassemblement national avait vocation à participer à un gouvernement. De quoi ajouter encore au désespoir des macronistes.</t>
+  </si>
+  <si>
+    <t>The news is huge, incredible and worrying. Yet it has gone virtually unnoticed. No debate, not the slightest comment in the press... And yet it's vital.
+Macron has run out of ideas... Yes, you read that right. Choupinet lacks inspiration. He no longer has a vision for the country. So much so that he organizes brainstorming sessions with his advisors. Le Point, which revealed the information in its February 16 edition, explains: “ The first meeting of this type took place on December 16, and the second a month later, on January 27 . One of the participants in these “ seminars ‘ confided to the weekly: ’ It's a chance to think hard about what's next, to reflect. The President goes fishing for ideas ”. You'd think he was dreaming! Why does he need to summon all his advisors - of whom there are some forty - to half-day brainstorming sessions?
+The man who in 2017 wanted to turn France into a “ start-up nation ” has had to scale back his ambitions. The Benalla affair, followed by the Gilets Jaunes crisis, forced him into the arena. His shocking, polemical little phrases like “ Les gens qui ne sont rien” ("People who are nothing ‘) or those ’ Gaulois refractory to change ‘ (’ Gaulois refractaires au changement ”) to talk about the French alienated him from the people, who found him arrogant and contemptuous. But that was before. During his first term. Youthful mistakes, so to speak.
+In the inaugural speech following his re-election on April 20, 2022, he presented himself as “ a new president (for) a new mandate ”. The Macron of 2022 would have nothing to do with the Macron of 2017. He had lots of plans for France. We were in for a treat! But then, ten months after his re-election, the dark clouds were gathering over his head. The pension reform is having trouble gaining public support, and MPs are squabbling in the Assembly.
+Macron's obsession
+It's not easy to pass legislation when you no longer have a real majority. Composing and negotiating with the opposition is not part of Macron's software. However, if you don't want to be condemned to stagnation, you have to do it. So, on the advice of Alexis Kohler, his Secretary General, who prepared the meetings, the Head of State turned to his advisors. His last faithful square? Faced with a situation he no longer masters, he needs to talk to them, question them, listen to them, note down their thoughts. For Macron has only one obsession in mind. How to prevent the country falling into the hands of the far right in 2027? This idea has been on his mind for months. So much so that news of his early resignation broke in the autumn. “ He doesn't want to be the one handing over the keys to the Élysée to Marine Le Pen in five years' time ,” confided a loyal supporter last October. It's a panic that has spread throughout the Macron family, right down to the members of parliament. During the stormy debates on pension reform, one of them had a waking nightmare as he watched Marine Le Pen. “ She stood there stoically. I suddenly saw her on the steps of the Élysée Palace. I'm afraid this is all going to end very badly...”.
+Faced with a panic-stricken majority and the bad manners and verbal outrages of the Nupes, the RN group in the Assembly offers an image of seriousness and responsibility. “ It's in the Assembly that the next presidential campaign is being prepared. I need a hand-picked army ,” confides Marine Le Pen in private. A winning strategy. According to a recent poll, the parliamentary group she chairs was the one most highly rated by the French during debates in the National Assembly. The former presidential runner-up and her party are gaining in credibility, especially on the right of the political spectrum. Last December, a survey by the Kantar institute showed that 40% of those polled thought that the Rassemblement National should be part of a government. All of which adds to the Macronists' despair.</t>
+  </si>
+  <si>
+    <t>La flambée des factures d’énergie menace de mettre six fabricants britanniques sur dix en faillite, selon une enquête qui met à nu l’ampleur de la crise à laquelle est confronté le prochain premier ministre.
+MakeUK, le groupe de lobbying des usines britanniques, a déclaré que près de la moitié des fabricants ont connu une hausse de plus de 100 % de leurs factures d’électricité au cours de l’année écoulée.
+« La crise actuelle place les entreprises devant un choix difficile », indique le rapport. « Réduire la production ou fermer carrément le magasin si l’aide n’arrive pas rapidement ».
+Le nom du nouveau Premier ministre britannique sera annoncé lundi, Liz Truss devant battre Rishi Sunak, son rival dans la course à la direction du Parti conservateur. Le gouvernement subit une pression intense pour annoncer des mesures de soutien plus large afin d’aider les consommateurs et les entreprises à faire face à une flambée sans précédent des coûts énergétiques mondiaux.
+Le secteur manufacturier britannique est déjà en déclin, selon un indice des directeurs d’achat publié par S&amp;P Global cette semaine. L’enquête de MakeUK indique que 13 % des usines ont désormais réduit leurs heures de fonctionnement ou évitent les périodes de pointe, tandis que 7 % arrêtent la production pendant de plus longues périodes.
+« Une action urgente est nécessaire de la part du nouveau gouvernement », a déclaré Stephen Phipson, directeur général de MakeUK. « Nous sommes déjà à la traîne par rapport à nos concurrents mondiaux ».</t>
+  </si>
+  <si>
+    <t>Soaring energy bills threaten to bankrupt six out of ten UK manufacturers, according to a survey that lays bare the scale of the crisis facing the next prime minister.
+MakeUK, the UK's factory lobbying group, said that almost half of manufacturers have experienced an increase of more than 100% in their electricity bills over the past year.
+“The current crisis presents companies with a difficult choice,” says the report. “Reduce production or close up store altogether if help doesn't arrive soon”.
+The name of Britain's new Prime Minister will be announced on Monday, with Liz Truss set to defeat Rishi Sunak, her rival in the Conservative Party leadership race. The government is under intense pressure to announce wider support measures to help consumers and businesses cope with an unprecedented surge in global energy costs.
+The UK manufacturing sector is already in decline, according to a purchasing managers' index published by S&amp;P Global this week. MakeUK's survey indicates that 13% of factories have now reduced their operating hours or are avoiding peak periods, while 7% are stopping production for longer periods.
+“Urgent action is needed from the new government,” said Stephen Phipson, Chief Executive of MakeUK. “We are already lagging behind our global competitors”.</t>
+  </si>
+  <si>
+    <t>Nos confrères de La Manche Libre racontent qu’un homme de 45 ans de nationalité algérienne a épousé à Cherbourg une Française alors qu’il était déjà marié en Algérie ! Il a été jugé par le tribunal judiciaire de Cherbourg le mardi 7 février. Pour son mariage en France, il a fourni de faux renseignements sur sa situation. Sa véritable épouse – algérienne- , avec laquelle il a deux enfants (!), a transmis aux autorités un courrier précisant la situation.
+À la barre, le mis en cause, décidément élégant, déclare ne pas la connaître ! Pourtant, un acte mentionne bien qu’il est marié depuis février 2007 en Algérie.
+En 2014, il a émis plusieurs demandes de visa pour venir en France ; or, sur les actes de naissance fournis lors de ces demandes, il est fait mention de son mariage en 2007.
+La procureure précise : “Il a fait usage d’un faux acte de naissance pour se marier en France. C’est une infraction grave.” Elle requiert douze mois de prison avec sursis, une inéligibilité de cinq ans et une interdiction de territoire français pendant dix ans.
+Compte tenu du dossier, le tribunal a prononcé la relaxe du prévenu le mardi 11 avril.</t>
+  </si>
+  <si>
+    <t>Our colleagues in La Manche Libre report that a 45-year-old man of Algerian nationality married a French woman in Cherbourg, even though he was already married in Algeria! He was tried by the Cherbourg judicial court on Tuesday February 7. For his marriage in France, he provided false information about his situation. His real Algerian wife, with whom he has two children (!), sent the authorities a letter clarifying the situation.
+On the stand, the accused, who is decidedly elegant, declares that he doesn't know her! However, a deed clearly states that he has been married in Algeria since February 2007.
+In 2014, he applied for several visas to come to France; however, the birth certificates provided with these applications mention his marriage in 2007.
+The prosecutor added: “He used a false birth certificate to get married in France. This is a serious offence. She requested a twelve-month suspended prison sentence, five years' ineligibility and a ten-year ban from French territory.
+In view of the case, the court acquitted the defendant on Tuesday April 11.</t>
   </si>
 </sst>
 </file>
@@ -404,7 +468,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="81.453125" customWidth="1"/>
@@ -444,6 +508,55 @@
         <v>6</v>
       </c>
     </row>
+    <row r="4" spans="1:3" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="362.5" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="246.5" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>